<commit_message>
update input function and add power constraint
</commit_message>
<xml_diff>
--- a/carbon_constraint.xlsx
+++ b/carbon_constraint.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hy4174/Documents/GitHub/GCAM_USA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4B99D84-BFD9-3340-81AB-B870A2A14E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0ADA38F-5F63-1941-99DE-A7B24E92894F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18300" yWindow="5760" windowWidth="27240" windowHeight="16440" xr2:uid="{CD997A8A-CBA1-F948-B390-49E2E92F265C}"/>
+    <workbookView xWindow="34600" yWindow="1840" windowWidth="26200" windowHeight="16440" xr2:uid="{CD997A8A-CBA1-F948-B390-49E2E92F265C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>scenario</t>
   </si>
@@ -66,13 +66,25 @@
   </si>
   <si>
     <t>stick + shock</t>
+  </si>
+  <si>
+    <t>trade base stick</t>
+  </si>
+  <si>
+    <t>2005 CO2 emission</t>
+  </si>
+  <si>
+    <t>EIA</t>
+  </si>
+  <si>
+    <t>Energy-Related Carbon Dioxide Emissions by State, 2005-2016</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -91,6 +103,13 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -114,10 +133,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F348AE-3E3A-F44A-97FA-98DAAA2E2B1D}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5" customWidth="1"/>
@@ -824,6 +844,55 @@
         <v>1141</v>
       </c>
     </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>10</v>
+      </c>
+      <c r="B30">
+        <f>5991*0.83</f>
+        <v>4972.53</v>
+      </c>
+      <c r="C30">
+        <f>5991*0.72</f>
+        <v>4313.5199999999995</v>
+      </c>
+      <c r="D30">
+        <f>5991*0.48</f>
+        <v>2875.68</v>
+      </c>
+      <c r="E30">
+        <f>0.34*5991</f>
+        <v>2036.94</v>
+      </c>
+      <c r="F30">
+        <f>E30-H32</f>
+        <v>1641.2933333333333</v>
+      </c>
+      <c r="G30">
+        <f>E30-H32*2</f>
+        <v>1245.6466666666665</v>
+      </c>
+      <c r="H30">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B32" t="s">
+        <v>12</v>
+      </c>
+      <c r="H32">
+        <f>(E30-H30)/3</f>
+        <v>395.6466666666667</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B33" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>